<commit_message>
Funcionalidades: imprimir_pedidos para vendedores y rol oficina
</commit_message>
<xml_diff>
--- a/excel/funcionalidades_maestro.xlsx
+++ b/excel/funcionalidades_maestro.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+  <workbookPr filterPrivacy="1"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
   </bookViews>
@@ -10,7 +10,7 @@
     <sheet name="Funcionalidades" sheetId="1" r:id="rId1"/>
     <sheet name="Roles" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="41">
   <si>
     <t>id</t>
   </si>
@@ -124,13 +124,31 @@
     <t>all</t>
   </si>
   <si>
-    <t>estado_de_cuentas</t>
+    <t>imprimir_pedidos</t>
+  </si>
+  <si>
+    <t>Imprimir pedidos</t>
+  </si>
+  <si>
+    <t>Bandeja de impresión de pedidos</t>
+  </si>
+  <si>
+    <t>🖨️</t>
+  </si>
+  <si>
+    <t>estado_de_cuentas,imprimir_pedidos</t>
+  </si>
+  <si>
+    <t>oficina</t>
+  </si>
+  <si>
+    <t>Oficina</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -466,7 +484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -559,6 +577,23 @@
         <v>9</v>
       </c>
     </row>
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -567,7 +602,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.140625" customWidth="1"/>
@@ -594,7 +629,7 @@
         <v>26</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -628,6 +663,17 @@
       </c>
       <c r="C5" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>